<commit_message>
feat(kontrak): ringkasan override pembayaran lalu, persen tagih, fix desa/kecamatan
- Placeholder desa/kecamatan pakai n_desa/n_kec
- Override persen tagih (100/95/5/30) dan multi pembayaran yang lalu
- Template ringkasan + POST export/preview ringkasan
</commit_message>
<xml_diff>
--- a/storage/app/templates/ringkasan_kontrak_template.xlsx
+++ b/storage/app/templates/ringkasan_kontrak_template.xlsx
@@ -21,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="[$-421]dd\ mmmm\ yyyy;@"/>
     <numFmt numFmtId="165" formatCode="&quot;Rp&quot;#,##0.00;\-&quot;Rp&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <name val="Aptos Narrow"/>
       <charset val="1"/>
@@ -47,12 +47,6 @@
     <font>
       <name val="Tahoma"/>
       <family val="2"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Tahoma"/>
-      <family val="2"/>
-      <color rgb="FFFF0000"/>
       <sz val="10"/>
     </font>
     <font>
@@ -133,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -214,10 +208,6 @@
       <alignment vertical="top"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="1" xfId="0">
       <alignment horizontal="left" vertical="top"/>
       <protection locked="0" hidden="0"/>
@@ -226,7 +216,7 @@
       <alignment horizontal="left" vertical="top"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -253,37 +243,37 @@
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="1" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="1" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -295,15 +285,15 @@
       <alignment horizontal="left" vertical="top"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -726,26 +716,26 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customFormat="1" customHeight="1" s="2">
-      <c r="A1" s="38" t="inlineStr">
+      <c r="A1" s="45" t="inlineStr">
         <is>
           <t>RINGKASAN KONTRAK</t>
         </is>
       </c>
     </row>
     <row r="2" ht="14.25" customFormat="1" customHeight="1" s="2">
-      <c r="A2" s="38" t="n"/>
-      <c r="B2" s="38" t="n"/>
-      <c r="C2" s="38" t="n"/>
-      <c r="D2" s="38" t="n"/>
-      <c r="E2" s="38" t="n"/>
-      <c r="F2" s="38" t="n"/>
-      <c r="G2" s="38" t="n"/>
-      <c r="H2" s="38" t="n"/>
-      <c r="I2" s="38" t="n"/>
-      <c r="J2" s="38" t="n"/>
-      <c r="K2" s="38" t="n"/>
-      <c r="L2" s="38" t="n"/>
-      <c r="M2" s="38" t="n"/>
+      <c r="A2" s="45" t="n"/>
+      <c r="B2" s="45" t="n"/>
+      <c r="C2" s="45" t="n"/>
+      <c r="D2" s="45" t="n"/>
+      <c r="E2" s="45" t="n"/>
+      <c r="F2" s="45" t="n"/>
+      <c r="G2" s="45" t="n"/>
+      <c r="H2" s="45" t="n"/>
+      <c r="I2" s="45" t="n"/>
+      <c r="J2" s="45" t="n"/>
+      <c r="K2" s="45" t="n"/>
+      <c r="L2" s="45" t="n"/>
+      <c r="M2" s="45" t="n"/>
     </row>
     <row r="3" customFormat="1" s="2">
       <c r="A3" s="3" t="n"/>
@@ -1018,7 +1008,7 @@
           <t>:</t>
         </is>
       </c>
-      <c r="E4" s="47" t="inlineStr">
+      <c r="E4" s="35" t="inlineStr">
         <is>
           <t xml:space="preserve">{check_dau} </t>
         </is>
@@ -1156,7 +1146,7 @@
       <c r="B10" s="4" t="n"/>
       <c r="C10" s="4" t="n"/>
       <c r="D10" s="4" t="n"/>
-      <c r="E10" s="47" t="inlineStr">
+      <c r="E10" s="35" t="inlineStr">
         <is>
           <t xml:space="preserve">{check_silpa} </t>
         </is>
@@ -1227,7 +1217,7 @@
       <c r="F13" s="5" t="n"/>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>{skpd}</t>
+          <t>Dinas Perumahan dan Kawasan Permukiman</t>
         </is>
       </c>
       <c r="H13" s="5" t="n"/>
@@ -1256,7 +1246,7 @@
       <c r="F14" s="5" t="n"/>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>{nomor_dpa}</t>
+          <t>900/Kep.09/BKAD/2/2026</t>
         </is>
       </c>
       <c r="H14" s="5" t="n"/>
@@ -1265,7 +1255,7 @@
       <c r="K14" s="10" t="n"/>
       <c r="L14" s="11" t="inlineStr">
         <is>
-          <t>Tanggal {tanggal_dpa}</t>
+          <t>Tanggal 03 Februari 2026</t>
         </is>
       </c>
       <c r="M14" s="5" t="n"/>
@@ -1289,7 +1279,7 @@
       <c r="F15" s="5" t="n"/>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t>{nama_program}</t>
+          <t>PROGRAM PENGELOLAAN DAN PENGEMBANGAN SISTEM PENYEDIAAN AIR MINUM</t>
         </is>
       </c>
       <c r="H15" s="5" t="n"/>
@@ -1316,17 +1306,17 @@
         </is>
       </c>
       <c r="F16" s="5" t="n"/>
-      <c r="G16" s="39" t="inlineStr">
+      <c r="G16" s="40" t="inlineStr">
         <is>
           <t>{nama_kegiatan}</t>
         </is>
       </c>
-      <c r="H16" s="48" t="n"/>
-      <c r="I16" s="48" t="n"/>
-      <c r="J16" s="48" t="n"/>
-      <c r="K16" s="48" t="n"/>
-      <c r="L16" s="48" t="n"/>
-      <c r="M16" s="48" t="n"/>
+      <c r="H16" s="47" t="n"/>
+      <c r="I16" s="47" t="n"/>
+      <c r="J16" s="47" t="n"/>
+      <c r="K16" s="47" t="n"/>
+      <c r="L16" s="47" t="n"/>
+      <c r="M16" s="47" t="n"/>
     </row>
     <row r="17" ht="30.75" customFormat="1" customHeight="1" s="2">
       <c r="A17" s="4" t="n">
@@ -1345,17 +1335,17 @@
         </is>
       </c>
       <c r="F17" s="5" t="n"/>
-      <c r="G17" s="40" t="inlineStr">
+      <c r="G17" s="41" t="inlineStr">
         <is>
           <t>{sub_kegiatan}</t>
         </is>
       </c>
-      <c r="H17" s="48" t="n"/>
-      <c r="I17" s="48" t="n"/>
-      <c r="J17" s="48" t="n"/>
-      <c r="K17" s="48" t="n"/>
-      <c r="L17" s="48" t="n"/>
-      <c r="M17" s="48" t="n"/>
+      <c r="H17" s="47" t="n"/>
+      <c r="I17" s="47" t="n"/>
+      <c r="J17" s="47" t="n"/>
+      <c r="K17" s="47" t="n"/>
+      <c r="L17" s="47" t="n"/>
+      <c r="M17" s="47" t="n"/>
     </row>
     <row r="18" ht="16.5" customFormat="1" customHeight="1" s="2" thickBot="1">
       <c r="A18" s="16" t="n">
@@ -1474,13 +1464,13 @@
         </is>
       </c>
       <c r="F21" s="5" t="n"/>
-      <c r="G21" s="49" t="inlineStr">
+      <c r="G21" s="48" t="inlineStr">
         <is>
           <t>{nilai_kontrak}</t>
         </is>
       </c>
-      <c r="H21" s="48" t="n"/>
-      <c r="I21" s="48" t="n"/>
+      <c r="H21" s="47" t="n"/>
+      <c r="I21" s="47" t="n"/>
       <c r="J21" s="5" t="n"/>
       <c r="K21" s="5" t="n"/>
       <c r="L21" s="5" t="n"/>
@@ -1501,14 +1491,14 @@
         </is>
       </c>
       <c r="F22" s="5" t="n"/>
-      <c r="G22" s="49" t="inlineStr">
+      <c r="G22" s="48" t="inlineStr">
         <is>
           <t>{nilai_kontrak_addendum}</t>
         </is>
       </c>
-      <c r="H22" s="48" t="n"/>
-      <c r="I22" s="48" t="n"/>
-      <c r="J22" s="48" t="n"/>
+      <c r="H22" s="47" t="n"/>
+      <c r="I22" s="47" t="n"/>
+      <c r="J22" s="47" t="n"/>
       <c r="K22" s="5" t="n"/>
       <c r="L22" s="5" t="n"/>
       <c r="M22" s="5" t="n"/>
@@ -1530,7 +1520,7 @@
         </is>
       </c>
       <c r="F23" s="5" t="n"/>
-      <c r="G23" s="23" t="inlineStr">
+      <c r="G23" s="46" t="inlineStr">
         <is>
           <t>{masa_hari_terbilang}</t>
         </is>
@@ -1557,13 +1547,13 @@
         </is>
       </c>
       <c r="F24" s="5" t="n"/>
-      <c r="G24" s="49" t="inlineStr">
-        <is>
-          <t>{masa_hari_addendum}</t>
-        </is>
-      </c>
-      <c r="H24" s="48" t="n"/>
-      <c r="I24" s="48" t="n"/>
+      <c r="G24" s="48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H24" s="47" t="n"/>
+      <c r="I24" s="47" t="n"/>
       <c r="J24" s="5" t="n"/>
       <c r="K24" s="5" t="n"/>
       <c r="L24" s="5" t="n"/>
@@ -1615,17 +1605,17 @@
         </is>
       </c>
       <c r="F26" s="5" t="n"/>
-      <c r="G26" s="24" t="inlineStr">
+      <c r="G26" s="23" t="inlineStr">
         <is>
           <t>{nama_penyedia} / {nama_direktur}</t>
         </is>
       </c>
-      <c r="H26" s="24" t="n"/>
-      <c r="I26" s="24" t="n"/>
-      <c r="J26" s="24" t="n"/>
-      <c r="K26" s="24" t="n"/>
-      <c r="L26" s="24" t="n"/>
-      <c r="M26" s="24" t="n"/>
+      <c r="H26" s="23" t="n"/>
+      <c r="I26" s="23" t="n"/>
+      <c r="J26" s="23" t="n"/>
+      <c r="K26" s="23" t="n"/>
+      <c r="L26" s="23" t="n"/>
+      <c r="M26" s="23" t="n"/>
     </row>
     <row r="27" ht="27.75" customFormat="1" customHeight="1" s="2">
       <c r="A27" s="4" t="n">
@@ -1644,17 +1634,17 @@
         </is>
       </c>
       <c r="F27" s="5" t="n"/>
-      <c r="G27" s="39" t="inlineStr">
+      <c r="G27" s="40" t="inlineStr">
         <is>
           <t>{alamat_penyedia}</t>
         </is>
       </c>
-      <c r="H27" s="48" t="n"/>
-      <c r="I27" s="48" t="n"/>
-      <c r="J27" s="48" t="n"/>
-      <c r="K27" s="48" t="n"/>
-      <c r="L27" s="48" t="n"/>
-      <c r="M27" s="48" t="n"/>
+      <c r="H27" s="47" t="n"/>
+      <c r="I27" s="47" t="n"/>
+      <c r="J27" s="47" t="n"/>
+      <c r="K27" s="47" t="n"/>
+      <c r="L27" s="47" t="n"/>
+      <c r="M27" s="47" t="n"/>
     </row>
     <row r="28" ht="16.5" customFormat="1" customHeight="1" s="2">
       <c r="A28" s="4" t="n">
@@ -1673,25 +1663,25 @@
         </is>
       </c>
       <c r="F28" s="5" t="n"/>
-      <c r="G28" s="25" t="inlineStr">
+      <c r="G28" s="24" t="inlineStr">
         <is>
           <t>{rekening_penyedia}</t>
         </is>
       </c>
-      <c r="H28" s="39" t="n"/>
-      <c r="I28" s="39" t="n"/>
-      <c r="J28" s="39" t="n"/>
-      <c r="K28" s="43" t="inlineStr">
+      <c r="H28" s="40" t="n"/>
+      <c r="I28" s="40" t="n"/>
+      <c r="J28" s="40" t="n"/>
+      <c r="K28" s="42" t="inlineStr">
         <is>
           <t>pada -</t>
         </is>
       </c>
-      <c r="L28" s="27" t="inlineStr">
+      <c r="L28" s="26" t="inlineStr">
         <is>
           <t>{bank_penyedia}</t>
         </is>
       </c>
-      <c r="M28" s="39" t="n"/>
+      <c r="M28" s="40" t="n"/>
     </row>
     <row r="29" ht="16.5" customFormat="1" customHeight="1" s="2">
       <c r="A29" s="4" t="n">
@@ -1710,17 +1700,17 @@
         </is>
       </c>
       <c r="F29" s="5" t="n"/>
-      <c r="G29" s="25" t="inlineStr">
+      <c r="G29" s="24" t="inlineStr">
         <is>
           <t>{npwp_penyedia}</t>
         </is>
       </c>
-      <c r="H29" s="39" t="n"/>
-      <c r="I29" s="39" t="n"/>
-      <c r="J29" s="39" t="n"/>
-      <c r="K29" s="39" t="n"/>
-      <c r="L29" s="39" t="n"/>
-      <c r="M29" s="39" t="n"/>
+      <c r="H29" s="40" t="n"/>
+      <c r="I29" s="40" t="n"/>
+      <c r="J29" s="40" t="n"/>
+      <c r="K29" s="40" t="n"/>
+      <c r="L29" s="40" t="n"/>
+      <c r="M29" s="40" t="n"/>
     </row>
     <row r="30" ht="24" customFormat="1" customHeight="1" s="2">
       <c r="A30" s="4" t="n">
@@ -1739,17 +1729,17 @@
         </is>
       </c>
       <c r="F30" s="5" t="n"/>
-      <c r="G30" s="40" t="inlineStr">
+      <c r="G30" s="41" t="inlineStr">
         <is>
           <t>{nama_paket}</t>
         </is>
       </c>
-      <c r="H30" s="48" t="n"/>
-      <c r="I30" s="48" t="n"/>
-      <c r="J30" s="48" t="n"/>
-      <c r="K30" s="48" t="n"/>
-      <c r="L30" s="48" t="n"/>
-      <c r="M30" s="48" t="n"/>
+      <c r="H30" s="47" t="n"/>
+      <c r="I30" s="47" t="n"/>
+      <c r="J30" s="47" t="n"/>
+      <c r="K30" s="47" t="n"/>
+      <c r="L30" s="47" t="n"/>
+      <c r="M30" s="47" t="n"/>
     </row>
     <row r="31" ht="19.5" customFormat="1" customHeight="1" s="2">
       <c r="A31" s="4" t="n"/>
@@ -1791,17 +1781,17 @@
         </is>
       </c>
       <c r="F32" s="5" t="n"/>
-      <c r="G32" s="39" t="inlineStr">
+      <c r="G32" s="40" t="inlineStr">
         <is>
           <t>Pembayaran dilakukan dengan cara</t>
         </is>
       </c>
-      <c r="H32" s="48" t="n"/>
-      <c r="I32" s="48" t="n"/>
-      <c r="J32" s="48" t="n"/>
-      <c r="K32" s="48" t="n"/>
-      <c r="L32" s="48" t="n"/>
-      <c r="M32" s="48" t="n"/>
+      <c r="H32" s="47" t="n"/>
+      <c r="I32" s="47" t="n"/>
+      <c r="J32" s="47" t="n"/>
+      <c r="K32" s="47" t="n"/>
+      <c r="L32" s="47" t="n"/>
+      <c r="M32" s="47" t="n"/>
     </row>
     <row r="33" ht="16.9" customFormat="1" customHeight="1" s="2">
       <c r="A33" s="4" t="n"/>
@@ -1814,17 +1804,17 @@
           <t>a.</t>
         </is>
       </c>
-      <c r="G33" s="43" t="inlineStr">
-        <is>
-          <t>{check_pembayaran_sekaligus} Sekaligus</t>
-        </is>
-      </c>
-      <c r="H33" s="48" t="n"/>
-      <c r="I33" s="48" t="n"/>
-      <c r="J33" s="48" t="n"/>
-      <c r="K33" s="48" t="n"/>
-      <c r="L33" s="48" t="n"/>
-      <c r="M33" s="48" t="n"/>
+      <c r="G33" s="42" t="inlineStr">
+        <is>
+          <t>Sekaligus</t>
+        </is>
+      </c>
+      <c r="H33" s="47" t="n"/>
+      <c r="I33" s="47" t="n"/>
+      <c r="J33" s="47" t="n"/>
+      <c r="K33" s="47" t="n"/>
+      <c r="L33" s="47" t="n"/>
+      <c r="M33" s="47" t="n"/>
     </row>
     <row r="34" ht="16.9" customFormat="1" customHeight="1" s="2">
       <c r="A34" s="4" t="n"/>
@@ -1837,17 +1827,17 @@
           <t>b.</t>
         </is>
       </c>
-      <c r="G34" s="43" t="inlineStr">
-        <is>
-          <t>{check_pembayaran_termin} Termin</t>
-        </is>
-      </c>
-      <c r="H34" s="48" t="n"/>
-      <c r="I34" s="48" t="n"/>
-      <c r="J34" s="48" t="n"/>
-      <c r="K34" s="48" t="n"/>
-      <c r="L34" s="48" t="n"/>
-      <c r="M34" s="48" t="n"/>
+      <c r="G34" s="42" t="inlineStr">
+        <is>
+          <t>Termin</t>
+        </is>
+      </c>
+      <c r="H34" s="47" t="n"/>
+      <c r="I34" s="47" t="n"/>
+      <c r="J34" s="47" t="n"/>
+      <c r="K34" s="47" t="n"/>
+      <c r="L34" s="47" t="n"/>
+      <c r="M34" s="47" t="n"/>
     </row>
     <row r="35" ht="16.9" customFormat="1" customHeight="1" s="2" thickBot="1">
       <c r="A35" s="16" t="n"/>
@@ -1860,17 +1850,17 @@
           <t>c.</t>
         </is>
       </c>
-      <c r="G35" s="44" t="inlineStr">
-        <is>
-          <t>{check_pembayaran_bulan} Bulan</t>
-        </is>
-      </c>
-      <c r="H35" s="50" t="n"/>
-      <c r="I35" s="50" t="n"/>
-      <c r="J35" s="50" t="n"/>
-      <c r="K35" s="50" t="n"/>
-      <c r="L35" s="50" t="n"/>
-      <c r="M35" s="50" t="n"/>
+      <c r="G35" s="43" t="inlineStr">
+        <is>
+          <t>Bulan</t>
+        </is>
+      </c>
+      <c r="H35" s="49" t="n"/>
+      <c r="I35" s="49" t="n"/>
+      <c r="J35" s="49" t="n"/>
+      <c r="K35" s="49" t="n"/>
+      <c r="L35" s="49" t="n"/>
+      <c r="M35" s="49" t="n"/>
     </row>
     <row r="36" ht="42" customFormat="1" customHeight="1" s="2">
       <c r="A36" s="4" t="n">
@@ -1887,15 +1877,15 @@
           <t>:</t>
         </is>
       </c>
-      <c r="F36" s="28" t="n"/>
-      <c r="G36" s="49" t="inlineStr">
+      <c r="F36" s="27" t="n"/>
+      <c r="G36" s="48" t="inlineStr">
         <is>
           <t>{nomor_jaminan_uang_muka}</t>
         </is>
       </c>
-      <c r="H36" s="48" t="n"/>
-      <c r="I36" s="48" t="n"/>
-      <c r="J36" s="29" t="n"/>
+      <c r="H36" s="47" t="n"/>
+      <c r="I36" s="47" t="n"/>
+      <c r="J36" s="28" t="n"/>
       <c r="K36" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">Tanggal </t>
@@ -1923,19 +1913,19 @@
           <t>:</t>
         </is>
       </c>
-      <c r="F37" s="28" t="n"/>
-      <c r="G37" s="37" t="inlineStr">
+      <c r="F37" s="27" t="n"/>
+      <c r="G37" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve"> {tgl_selesai}</t>
         </is>
       </c>
-      <c r="H37" s="48" t="n"/>
-      <c r="I37" s="48" t="n"/>
-      <c r="J37" s="48" t="n"/>
-      <c r="K37" s="48" t="n"/>
-      <c r="L37" s="48" t="n"/>
-      <c r="M37" s="48" t="n"/>
-      <c r="N37" s="48" t="n"/>
+      <c r="H37" s="47" t="n"/>
+      <c r="I37" s="47" t="n"/>
+      <c r="J37" s="47" t="n"/>
+      <c r="K37" s="47" t="n"/>
+      <c r="L37" s="47" t="n"/>
+      <c r="M37" s="47" t="n"/>
+      <c r="N37" s="47" t="n"/>
     </row>
     <row r="38" ht="21" customFormat="1" customHeight="1" s="2">
       <c r="A38" s="4" t="n">
@@ -1952,15 +1942,15 @@
           <t>:</t>
         </is>
       </c>
-      <c r="F38" s="28" t="n"/>
-      <c r="G38" s="31" t="inlineStr">
+      <c r="F38" s="27" t="n"/>
+      <c r="G38" s="30" t="inlineStr">
         <is>
           <t>{nomor_bastp}</t>
         </is>
       </c>
-      <c r="H38" s="29" t="n"/>
-      <c r="I38" s="29" t="n"/>
-      <c r="J38" s="29" t="n"/>
+      <c r="H38" s="28" t="n"/>
+      <c r="I38" s="28" t="n"/>
+      <c r="J38" s="28" t="n"/>
       <c r="K38" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">Tanggal </t>
@@ -1971,13 +1961,13 @@
           <t>{tgl_bastp}</t>
         </is>
       </c>
-      <c r="M38" s="29" t="n"/>
+      <c r="M38" s="28" t="n"/>
     </row>
     <row r="39" customFormat="1" s="2">
       <c r="A39" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="B39" s="45" t="inlineStr">
+      <c r="B39" s="37" t="inlineStr">
         <is>
           <t>Jangka Waktu Pemeliharaan</t>
         </is>
@@ -1987,10 +1977,10 @@
           <t>:</t>
         </is>
       </c>
-      <c r="F39" s="28" t="n"/>
+      <c r="F39" s="27" t="n"/>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>{jangka_pemeliharaan}</t>
+          <t>180 (seratus delapan puluh) Hari Kalender</t>
         </is>
       </c>
       <c r="H39" s="5" t="n"/>
@@ -2004,7 +1994,7 @@
       <c r="A40" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="B40" s="45" t="inlineStr">
+      <c r="B40" s="37" t="inlineStr">
         <is>
           <t>Tanggal Waktu Pemeliharaan</t>
         </is>
@@ -2014,7 +2004,7 @@
           <t>:</t>
         </is>
       </c>
-      <c r="F40" s="28" t="n"/>
+      <c r="F40" s="27" t="n"/>
       <c r="G40" s="12" t="inlineStr">
         <is>
           <t>{mulai_selesai_pemeliharaan}</t>
@@ -2042,27 +2032,27 @@
           <t>:</t>
         </is>
       </c>
-      <c r="F41" s="28" t="n"/>
-      <c r="G41" s="49" t="inlineStr">
+      <c r="F41" s="27" t="n"/>
+      <c r="G41" s="48" t="inlineStr">
         <is>
           <t>{nomor_jaminan_pemeliharaan}</t>
         </is>
       </c>
-      <c r="H41" s="48" t="n"/>
-      <c r="I41" s="48" t="n"/>
-      <c r="J41" s="29" t="n"/>
+      <c r="H41" s="47" t="n"/>
+      <c r="I41" s="47" t="n"/>
+      <c r="J41" s="28" t="n"/>
       <c r="K41" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">Tanggal </t>
         </is>
       </c>
-      <c r="L41" s="49" t="inlineStr">
+      <c r="L41" s="48" t="inlineStr">
         <is>
           <t>{tanggal_jaminan_pemeliharaan}</t>
         </is>
       </c>
-      <c r="M41" s="48" t="n"/>
-      <c r="N41" s="48" t="n"/>
+      <c r="M41" s="47" t="n"/>
+      <c r="N41" s="47" t="n"/>
     </row>
     <row r="42" ht="21" customFormat="1" customHeight="1" s="2">
       <c r="A42" s="4" t="n">
@@ -2079,15 +2069,15 @@
           <t>:</t>
         </is>
       </c>
-      <c r="F42" s="28" t="n"/>
-      <c r="G42" s="31" t="inlineStr">
-        <is>
-          <t>{nomor_bastp}</t>
-        </is>
-      </c>
-      <c r="H42" s="29" t="n"/>
-      <c r="I42" s="29" t="n"/>
-      <c r="J42" s="29" t="n"/>
+      <c r="F42" s="27" t="n"/>
+      <c r="G42" s="30" t="inlineStr">
+        <is>
+          <t>{nomor_bastp_95}</t>
+        </is>
+      </c>
+      <c r="H42" s="28" t="n"/>
+      <c r="I42" s="28" t="n"/>
+      <c r="J42" s="28" t="n"/>
       <c r="K42" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">Tanggal </t>
@@ -2095,10 +2085,10 @@
       </c>
       <c r="L42" s="21" t="inlineStr">
         <is>
-          <t>{tgl_bastp}</t>
-        </is>
-      </c>
-      <c r="M42" s="29" t="n"/>
+          <t>{tgl_bastp_95}</t>
+        </is>
+      </c>
+      <c r="M42" s="28" t="n"/>
     </row>
     <row r="43" ht="18" customFormat="1" customHeight="1" s="2">
       <c r="A43" s="4" t="n">
@@ -2115,8 +2105,8 @@
           <t>:</t>
         </is>
       </c>
-      <c r="F43" s="28" t="n"/>
-      <c r="G43" s="31" t="inlineStr">
+      <c r="F43" s="27" t="n"/>
+      <c r="G43" s="30" t="inlineStr">
         <is>
           <t>{nomor_bap}</t>
         </is>
@@ -2129,7 +2119,7 @@
           <t xml:space="preserve">Tanggal </t>
         </is>
       </c>
-      <c r="L43" s="37" t="inlineStr">
+      <c r="L43" s="44" t="inlineStr">
         <is>
           <t>{tgl_bap}</t>
         </is>
@@ -2151,18 +2141,18 @@
           <t>:</t>
         </is>
       </c>
-      <c r="F44" s="28" t="n"/>
-      <c r="G44" s="49" t="inlineStr">
-        <is>
-          <t>{nilai_kontrak_5persen}</t>
-        </is>
-      </c>
-      <c r="H44" s="48" t="n"/>
-      <c r="I44" s="48" t="n"/>
+      <c r="F44" s="27" t="n"/>
+      <c r="G44" s="48" t="inlineStr">
+        <is>
+          <t>{nilai_tagih}</t>
+        </is>
+      </c>
+      <c r="H44" s="47" t="n"/>
+      <c r="I44" s="47" t="n"/>
       <c r="J44" s="5" t="n"/>
       <c r="K44" s="10" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>{persen_tagih}</t>
         </is>
       </c>
       <c r="L44" s="5" t="inlineStr">
@@ -2187,18 +2177,18 @@
           <t>:</t>
         </is>
       </c>
-      <c r="F45" s="28" t="inlineStr">
+      <c r="F45" s="27" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G45" s="49" t="inlineStr">
-        <is>
-          <t>Uang Muka</t>
-        </is>
-      </c>
-      <c r="H45" s="49" t="n"/>
-      <c r="I45" s="49" t="n"/>
+      <c r="G45" s="48" t="inlineStr">
+        <is>
+          <t>{pembayaran_lalu_1_jenis}</t>
+        </is>
+      </c>
+      <c r="H45" s="48" t="n"/>
+      <c r="I45" s="48" t="n"/>
       <c r="J45" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">Tanggal </t>
@@ -2206,12 +2196,12 @@
       </c>
       <c r="K45" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>{pembayaran_lalu_1_tanggal}</t>
         </is>
       </c>
       <c r="L45" s="5" t="inlineStr">
         <is>
-          <t>Rp -</t>
+          <t>{pembayaran_lalu_1_nominal}</t>
         </is>
       </c>
       <c r="M45" s="5" t="n"/>
@@ -2221,18 +2211,18 @@
       <c r="B46" s="4" t="n"/>
       <c r="C46" s="4" t="n"/>
       <c r="E46" s="8" t="n"/>
-      <c r="F46" s="28" t="inlineStr">
+      <c r="F46" s="27" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G46" s="49" t="inlineStr">
-        <is>
-          <t>MC / Termin I</t>
-        </is>
-      </c>
-      <c r="H46" s="49" t="n"/>
-      <c r="I46" s="49" t="n"/>
+      <c r="G46" s="48" t="inlineStr">
+        <is>
+          <t>{pembayaran_lalu_2_jenis}</t>
+        </is>
+      </c>
+      <c r="H46" s="48" t="n"/>
+      <c r="I46" s="48" t="n"/>
       <c r="J46" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">Tanggal </t>
@@ -2240,12 +2230,12 @@
       </c>
       <c r="K46" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>{pembayaran_lalu_2_tanggal}</t>
         </is>
       </c>
       <c r="L46" s="5" t="inlineStr">
         <is>
-          <t>Rp -</t>
+          <t>{pembayaran_lalu_2_nominal}</t>
         </is>
       </c>
       <c r="M46" s="5" t="n"/>
@@ -2255,18 +2245,18 @@
       <c r="B47" s="4" t="n"/>
       <c r="C47" s="4" t="n"/>
       <c r="E47" s="8" t="n"/>
-      <c r="F47" s="28" t="inlineStr">
+      <c r="F47" s="27" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G47" s="49" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H47" s="49" t="n"/>
-      <c r="I47" s="49" t="n"/>
+      <c r="G47" s="48" t="inlineStr">
+        <is>
+          <t>{pembayaran_lalu_3_jenis}</t>
+        </is>
+      </c>
+      <c r="H47" s="48" t="n"/>
+      <c r="I47" s="48" t="n"/>
       <c r="J47" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">Tanggal </t>
@@ -2274,12 +2264,12 @@
       </c>
       <c r="K47" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>{pembayaran_lalu_3_tanggal}</t>
         </is>
       </c>
       <c r="L47" s="5" t="inlineStr">
         <is>
-          <t>Rp -</t>
+          <t>{pembayaran_lalu_3_nominal}</t>
         </is>
       </c>
       <c r="M47" s="5" t="n"/>
@@ -2300,7 +2290,7 @@
         </is>
       </c>
       <c r="F48" s="7" t="n"/>
-      <c r="G48" s="31" t="inlineStr">
+      <c r="G48" s="30" t="inlineStr">
         <is>
           <t>{nama_pptk}</t>
         </is>
@@ -2313,7 +2303,7 @@
           <t>NIP</t>
         </is>
       </c>
-      <c r="L48" s="31" t="inlineStr">
+      <c r="L48" s="30" t="inlineStr">
         <is>
           <t>{nip_pptk}</t>
         </is>
@@ -2335,18 +2325,18 @@
           <t>:</t>
         </is>
       </c>
-      <c r="F49" s="28" t="n"/>
-      <c r="G49" s="42" t="inlineStr">
+      <c r="F49" s="27" t="n"/>
+      <c r="G49" s="39" t="inlineStr">
         <is>
           <t>Denda merupakan sanksi finansial yang dikenakan kepada Penyedia, sedangkan ganti rugi merupakan sanksi finansial yang dikenakan kepada PPK, karena terjadinya cedera janji/ wanprestasi yang tercantum dalam kontrak</t>
         </is>
       </c>
-      <c r="H49" s="48" t="n"/>
-      <c r="I49" s="48" t="n"/>
-      <c r="J49" s="48" t="n"/>
-      <c r="K49" s="48" t="n"/>
-      <c r="L49" s="48" t="n"/>
-      <c r="M49" s="48" t="n"/>
+      <c r="H49" s="47" t="n"/>
+      <c r="I49" s="47" t="n"/>
+      <c r="J49" s="47" t="n"/>
+      <c r="K49" s="47" t="n"/>
+      <c r="L49" s="47" t="n"/>
+      <c r="M49" s="47" t="n"/>
     </row>
     <row r="50" ht="18.6" customFormat="1" customHeight="1" s="2">
       <c r="A50" s="4" t="n"/>
@@ -2354,7 +2344,7 @@
       <c r="D50" s="4" t="n"/>
       <c r="E50" s="8" t="n"/>
       <c r="F50" s="4" t="n"/>
-      <c r="G50" s="41" t="n"/>
+      <c r="G50" s="38" t="n"/>
     </row>
     <row r="51" ht="18" customFormat="1" customHeight="1" s="2">
       <c r="A51" s="4" t="n"/>
@@ -2367,7 +2357,7 @@
       <c r="D51" s="4" t="n"/>
       <c r="E51" s="8" t="n"/>
       <c r="F51" s="4" t="n"/>
-      <c r="G51" s="32" t="n"/>
+      <c r="G51" s="31" t="n"/>
       <c r="H51" s="4" t="n"/>
       <c r="I51" s="4" t="n"/>
       <c r="J51" s="4" t="n"/>
@@ -2382,7 +2372,7 @@
       <c r="D52" s="4" t="n"/>
       <c r="E52" s="8" t="n"/>
       <c r="F52" s="4" t="n"/>
-      <c r="G52" s="32" t="n"/>
+      <c r="G52" s="31" t="n"/>
       <c r="H52" s="4" t="n"/>
       <c r="I52" s="4" t="n"/>
       <c r="J52" s="4" t="n"/>
@@ -2401,8 +2391,8 @@
       <c r="H53" s="5" t="n"/>
       <c r="I53" s="5" t="n"/>
       <c r="J53" s="5" t="n"/>
-      <c r="K53" s="28" t="n"/>
-      <c r="L53" s="33" t="inlineStr">
+      <c r="K53" s="27" t="n"/>
+      <c r="L53" s="32" t="inlineStr">
         <is>
           <t>Cianjur, ….................</t>
         </is>
@@ -2663,8 +2653,8 @@
       <c r="H54" s="5" t="n"/>
       <c r="I54" s="5" t="n"/>
       <c r="J54" s="5" t="n"/>
-      <c r="K54" s="28" t="n"/>
-      <c r="L54" s="33" t="n"/>
+      <c r="K54" s="27" t="n"/>
+      <c r="L54" s="32" t="n"/>
       <c r="M54" s="5" t="n"/>
       <c r="N54" s="3" t="n"/>
       <c r="O54" s="3" t="n"/>
@@ -2913,7 +2903,7 @@
     <row r="55" customFormat="1" s="2">
       <c r="A55" s="4" t="n"/>
       <c r="B55" s="4" t="n"/>
-      <c r="C55" s="33" t="inlineStr">
+      <c r="C55" s="32" t="inlineStr">
         <is>
           <t>Penyedia,</t>
         </is>
@@ -2925,8 +2915,8 @@
       <c r="H55" s="5" t="n"/>
       <c r="I55" s="5" t="n"/>
       <c r="J55" s="5" t="n"/>
-      <c r="K55" s="28" t="n"/>
-      <c r="L55" s="33" t="inlineStr">
+      <c r="K55" s="27" t="n"/>
+      <c r="L55" s="32" t="inlineStr">
         <is>
           <t>Pejabat Pembuat Komitmen,</t>
         </is>
@@ -3179,7 +3169,7 @@
     <row r="56" customFormat="1" s="2">
       <c r="A56" s="4" t="n"/>
       <c r="B56" s="4" t="n"/>
-      <c r="C56" s="33" t="inlineStr">
+      <c r="C56" s="32" t="inlineStr">
         <is>
           <t>{nama_penyedia}</t>
         </is>
@@ -3191,8 +3181,8 @@
       <c r="H56" s="5" t="n"/>
       <c r="I56" s="5" t="n"/>
       <c r="J56" s="5" t="n"/>
-      <c r="K56" s="28" t="n"/>
-      <c r="L56" s="33" t="n"/>
+      <c r="K56" s="27" t="n"/>
+      <c r="L56" s="32" t="n"/>
       <c r="M56" s="5" t="n"/>
       <c r="N56" s="3" t="n"/>
       <c r="O56" s="3" t="n"/>
@@ -3449,8 +3439,8 @@
       <c r="H57" s="5" t="n"/>
       <c r="I57" s="5" t="n"/>
       <c r="J57" s="5" t="n"/>
-      <c r="K57" s="28" t="n"/>
-      <c r="L57" s="33" t="n"/>
+      <c r="K57" s="27" t="n"/>
+      <c r="L57" s="32" t="n"/>
       <c r="M57" s="5" t="n"/>
       <c r="N57" s="3" t="n"/>
       <c r="O57" s="3" t="n"/>
@@ -3707,7 +3697,7 @@
       <c r="H58" s="5" t="n"/>
       <c r="I58" s="5" t="n"/>
       <c r="J58" s="5" t="n"/>
-      <c r="K58" s="28" t="n"/>
+      <c r="K58" s="27" t="n"/>
       <c r="L58" s="5" t="n"/>
       <c r="M58" s="5" t="n"/>
       <c r="N58" s="3" t="n"/>
@@ -3965,7 +3955,7 @@
       <c r="H59" s="5" t="n"/>
       <c r="I59" s="5" t="n"/>
       <c r="J59" s="5" t="n"/>
-      <c r="K59" s="28" t="n"/>
+      <c r="K59" s="27" t="n"/>
       <c r="L59" s="5" t="n"/>
       <c r="M59" s="5" t="n"/>
       <c r="N59" s="3" t="n"/>
@@ -4223,7 +4213,7 @@
       <c r="H60" s="5" t="n"/>
       <c r="I60" s="5" t="n"/>
       <c r="J60" s="5" t="n"/>
-      <c r="K60" s="28" t="n"/>
+      <c r="K60" s="27" t="n"/>
       <c r="L60" s="5" t="n"/>
       <c r="M60" s="5" t="n"/>
       <c r="N60" s="3" t="n"/>
@@ -4473,7 +4463,7 @@
     <row r="61" customFormat="1" s="2">
       <c r="A61" s="4" t="n"/>
       <c r="B61" s="4" t="n"/>
-      <c r="C61" s="46" t="inlineStr">
+      <c r="C61" s="34" t="inlineStr">
         <is>
           <t>{nama_direktur}</t>
         </is>
@@ -4485,7 +4475,7 @@
       <c r="H61" s="5" t="n"/>
       <c r="I61" s="5" t="n"/>
       <c r="J61" s="5" t="n"/>
-      <c r="K61" s="28" t="n"/>
+      <c r="K61" s="27" t="n"/>
       <c r="L61" s="34" t="inlineStr">
         <is>
           <t>{nama_ppk}</t>
@@ -4739,7 +4729,7 @@
     <row r="62" ht="18" customFormat="1" customHeight="1" s="2">
       <c r="A62" s="4" t="n"/>
       <c r="B62" s="4" t="n"/>
-      <c r="C62" s="33" t="inlineStr">
+      <c r="C62" s="32" t="inlineStr">
         <is>
           <t>Direktur</t>
         </is>
@@ -4748,13 +4738,13 @@
       <c r="E62" s="5" t="n"/>
       <c r="F62" s="5" t="n"/>
       <c r="G62" s="5" t="n"/>
-      <c r="H62" s="35" t="n"/>
+      <c r="H62" s="33" t="n"/>
       <c r="I62" s="5" t="n"/>
       <c r="J62" s="5" t="n"/>
-      <c r="K62" s="28" t="n"/>
-      <c r="L62" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="K62" s="27" t="n"/>
+      <c r="L62" s="32" t="inlineStr">
+        <is>
+          <t>{nip_ppk}</t>
         </is>
       </c>
       <c r="M62" s="5" t="n"/>
@@ -4762,17 +4752,17 @@
     <row r="63" customFormat="1" s="2">
       <c r="A63" s="3" t="n"/>
       <c r="B63" s="3" t="n"/>
-      <c r="C63" s="28" t="n"/>
-      <c r="D63" s="28" t="n"/>
-      <c r="E63" s="28" t="n"/>
-      <c r="F63" s="28" t="n"/>
-      <c r="G63" s="28" t="n"/>
-      <c r="H63" s="28" t="n"/>
-      <c r="I63" s="28" t="n"/>
-      <c r="J63" s="28" t="n"/>
-      <c r="K63" s="28" t="n"/>
-      <c r="L63" s="28" t="n"/>
-      <c r="M63" s="28" t="n"/>
+      <c r="C63" s="27" t="n"/>
+      <c r="D63" s="27" t="n"/>
+      <c r="E63" s="27" t="n"/>
+      <c r="F63" s="27" t="n"/>
+      <c r="G63" s="27" t="n"/>
+      <c r="H63" s="27" t="n"/>
+      <c r="I63" s="27" t="n"/>
+      <c r="J63" s="27" t="n"/>
+      <c r="K63" s="27" t="n"/>
+      <c r="L63" s="27" t="n"/>
+      <c r="M63" s="27" t="n"/>
       <c r="N63" s="3" t="n"/>
       <c r="O63" s="3" t="n"/>
       <c r="P63" s="3" t="n"/>

</xml_diff>